<commit_message>
feat: Add MASTER_ADMIN role and permanent delete functionality
- Add MASTER_ADMIN role to RBAC system with full permissions
- Update admin@bbq.com to MASTER_ADMIN in seed
- Add role management API (/api/admin/users/[id])
- Add permanent delete API (/api/manuals/[id]/permanent-delete)
- Add batch permanent delete API (/api/manuals/batch-permanent-delete)
- Update admin page with dynamic role assignment
- Add permanent delete buttons in Archive tab for Master Admin
- Fix ESLint configuration for Next.js 14 compatibility
- Downgrade ESLint to v8 for compatibility with eslint-config-next
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29705"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D946FE1-4524-473E-988F-37EE13A85115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A489AFDF-1607-425E-A1AA-024DF6AAE4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="현재 템플릿" sheetId="1" r:id="rId1"/>
@@ -217,7 +217,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;_-;_-@"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;_-;_-@"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -1075,7 +1075,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1097,6 +1097,181 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1107,179 +1282,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1636,130 +1639,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
     </row>
     <row r="2" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
     </row>
     <row r="3" spans="2:10" ht="18" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="15"/>
+      <c r="J3" s="80"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="81"/>
+      <c r="E5" s="81"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="81"/>
+      <c r="H5" s="81"/>
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="B6" s="81"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="81"/>
+      <c r="F6" s="81"/>
+      <c r="G6" s="81"/>
+      <c r="H6" s="81"/>
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="B7" s="81"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="81"/>
+      <c r="E7" s="81"/>
+      <c r="F7" s="81"/>
+      <c r="G7" s="81"/>
+      <c r="H7" s="81"/>
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="81"/>
+      <c r="D8" s="81"/>
+      <c r="E8" s="81"/>
+      <c r="F8" s="81"/>
+      <c r="G8" s="81"/>
+      <c r="H8" s="81"/>
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="81"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="81"/>
+      <c r="H9" s="81"/>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="81"/>
+      <c r="D10" s="81"/>
+      <c r="E10" s="81"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="81"/>
+      <c r="H10" s="81"/>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+      <c r="B11" s="81"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="81"/>
+      <c r="G11" s="81"/>
+      <c r="H11" s="81"/>
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="2:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
       <c r="E12" s="4" t="s">
         <v>7</v>
       </c>
@@ -2077,665 +2080,665 @@
       <c r="J31" s="12"/>
     </row>
     <row r="32" spans="2:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
+      <c r="C32" s="83"/>
+      <c r="D32" s="83"/>
+      <c r="E32" s="83"/>
+      <c r="F32" s="83"/>
+      <c r="G32" s="83"/>
+      <c r="H32" s="83"/>
+      <c r="I32" s="83"/>
+      <c r="J32" s="83"/>
     </row>
     <row r="33" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
+      <c r="C33" s="75"/>
+      <c r="D33" s="75"/>
+      <c r="E33" s="75"/>
+      <c r="F33" s="75"/>
+      <c r="G33" s="75"/>
+      <c r="H33" s="75"/>
+      <c r="I33" s="75"/>
+      <c r="J33" s="75"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="21" t="s">
+      <c r="C34" s="76"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
-    </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
+      <c r="I34" s="77"/>
+      <c r="J34" s="77"/>
+    </row>
+    <row r="35" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="6"/>
-      <c r="E35" s="22" t="s">
+      <c r="E35" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="56"/>
+      <c r="J35" s="56"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="6"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="56"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" s="6"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="56"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" s="6"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="56"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" s="6"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" s="6"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="56"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" s="6"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="56"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" s="6"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" s="6"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="56"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" s="6"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="22"/>
-      <c r="I44" s="22"/>
-      <c r="J44" s="22"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="56"/>
+      <c r="G44" s="56"/>
+      <c r="H44" s="56"/>
+      <c r="I44" s="56"/>
+      <c r="J44" s="56"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" s="6"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="56"/>
+      <c r="H45" s="56"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="56"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" s="6"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
+      <c r="E46" s="56"/>
+      <c r="F46" s="56"/>
+      <c r="G46" s="56"/>
+      <c r="H46" s="56"/>
+      <c r="I46" s="56"/>
+      <c r="J46" s="56"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" s="6"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="22"/>
-      <c r="J47" s="22"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="56"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="56"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" s="6"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="56"/>
+      <c r="J48" s="56"/>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" s="6"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22"/>
-      <c r="J49" s="22"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="56"/>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" s="6"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="56"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="56"/>
+      <c r="I50" s="56"/>
+      <c r="J50" s="56"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51" s="6"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="56"/>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B52" s="6"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22"/>
-      <c r="J52" s="22"/>
+      <c r="E52" s="56"/>
+      <c r="F52" s="56"/>
+      <c r="G52" s="56"/>
+      <c r="H52" s="56"/>
+      <c r="I52" s="56"/>
+      <c r="J52" s="56"/>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" s="6"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
+      <c r="E53" s="56"/>
+      <c r="F53" s="56"/>
+      <c r="G53" s="56"/>
+      <c r="H53" s="56"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="6"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="22"/>
-      <c r="H54" s="22"/>
-      <c r="I54" s="22"/>
-      <c r="J54" s="22"/>
+      <c r="E54" s="56"/>
+      <c r="F54" s="56"/>
+      <c r="G54" s="56"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="56"/>
+      <c r="J54" s="56"/>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55" s="6"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="22"/>
-      <c r="I55" s="22"/>
-      <c r="J55" s="22"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="56"/>
+      <c r="H55" s="56"/>
+      <c r="I55" s="56"/>
+      <c r="J55" s="56"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56" s="6"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="22"/>
-      <c r="I56" s="22"/>
-      <c r="J56" s="22"/>
+      <c r="E56" s="56"/>
+      <c r="F56" s="56"/>
+      <c r="G56" s="56"/>
+      <c r="H56" s="56"/>
+      <c r="I56" s="56"/>
+      <c r="J56" s="56"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57" s="6"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="22"/>
-      <c r="I57" s="22"/>
-      <c r="J57" s="22"/>
+      <c r="E57" s="56"/>
+      <c r="F57" s="56"/>
+      <c r="G57" s="56"/>
+      <c r="H57" s="56"/>
+      <c r="I57" s="56"/>
+      <c r="J57" s="56"/>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B58" s="6"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="22"/>
-      <c r="I58" s="22"/>
-      <c r="J58" s="22"/>
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
+      <c r="I58" s="56"/>
+      <c r="J58" s="56"/>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="6"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
+      <c r="E59" s="56"/>
+      <c r="F59" s="56"/>
+      <c r="G59" s="56"/>
+      <c r="H59" s="56"/>
+      <c r="I59" s="56"/>
+      <c r="J59" s="56"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60" s="6"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="56"/>
+      <c r="G60" s="56"/>
+      <c r="H60" s="56"/>
+      <c r="I60" s="56"/>
+      <c r="J60" s="56"/>
     </row>
     <row r="61" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B61" s="6"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
+      <c r="E61" s="56"/>
+      <c r="F61" s="56"/>
+      <c r="G61" s="56"/>
+      <c r="H61" s="56"/>
+      <c r="I61" s="56"/>
+      <c r="J61" s="56"/>
     </row>
     <row r="62" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B62" s="6"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
+      <c r="E62" s="56"/>
+      <c r="F62" s="56"/>
+      <c r="G62" s="56"/>
+      <c r="H62" s="56"/>
+      <c r="I62" s="56"/>
+      <c r="J62" s="56"/>
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B63" s="6"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="22"/>
-      <c r="I63" s="22"/>
-      <c r="J63" s="22"/>
+      <c r="E63" s="56"/>
+      <c r="F63" s="56"/>
+      <c r="G63" s="56"/>
+      <c r="H63" s="56"/>
+      <c r="I63" s="56"/>
+      <c r="J63" s="56"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64" s="6"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="22"/>
+      <c r="E64" s="56"/>
+      <c r="F64" s="56"/>
+      <c r="G64" s="56"/>
+      <c r="H64" s="56"/>
+      <c r="I64" s="56"/>
+      <c r="J64" s="56"/>
     </row>
     <row r="65" spans="2:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="18"/>
-      <c r="D65" s="18"/>
-      <c r="E65" s="18"/>
-      <c r="F65" s="18"/>
-      <c r="G65" s="18"/>
-      <c r="H65" s="18"/>
-      <c r="I65" s="18"/>
-      <c r="J65" s="18"/>
+      <c r="C65" s="74"/>
+      <c r="D65" s="74"/>
+      <c r="E65" s="74"/>
+      <c r="F65" s="74"/>
+      <c r="G65" s="74"/>
+      <c r="H65" s="74"/>
+      <c r="I65" s="74"/>
+      <c r="J65" s="74"/>
     </row>
     <row r="66" spans="2:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="19" t="s">
+      <c r="B66" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="19"/>
-      <c r="D66" s="19"/>
-      <c r="E66" s="19"/>
-      <c r="F66" s="19"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="19"/>
-      <c r="I66" s="19"/>
-      <c r="J66" s="19"/>
+      <c r="C66" s="75"/>
+      <c r="D66" s="75"/>
+      <c r="E66" s="75"/>
+      <c r="F66" s="75"/>
+      <c r="G66" s="75"/>
+      <c r="H66" s="75"/>
+      <c r="I66" s="75"/>
+      <c r="J66" s="75"/>
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B67" s="20" t="s">
+      <c r="B67" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="C67" s="20"/>
-      <c r="D67" s="20"/>
-      <c r="E67" s="21" t="s">
+      <c r="C67" s="76"/>
+      <c r="D67" s="76"/>
+      <c r="E67" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="F67" s="21"/>
-      <c r="G67" s="21"/>
-      <c r="H67" s="21"/>
-      <c r="I67" s="21"/>
-      <c r="J67" s="21"/>
-    </row>
-    <row r="68" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="F67" s="77"/>
+      <c r="G67" s="77"/>
+      <c r="H67" s="77"/>
+      <c r="I67" s="77"/>
+      <c r="J67" s="77"/>
+    </row>
+    <row r="68" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="6"/>
-      <c r="E68" s="22" t="s">
+      <c r="E68" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="22"/>
-      <c r="I68" s="22"/>
-      <c r="J68" s="22"/>
+      <c r="F68" s="56"/>
+      <c r="G68" s="56"/>
+      <c r="H68" s="56"/>
+      <c r="I68" s="56"/>
+      <c r="J68" s="56"/>
     </row>
     <row r="69" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B69" s="6"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
+      <c r="E69" s="56"/>
+      <c r="F69" s="56"/>
+      <c r="G69" s="56"/>
+      <c r="H69" s="56"/>
+      <c r="I69" s="56"/>
+      <c r="J69" s="56"/>
     </row>
     <row r="70" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B70" s="6"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="22"/>
+      <c r="E70" s="56"/>
+      <c r="F70" s="56"/>
+      <c r="G70" s="56"/>
+      <c r="H70" s="56"/>
+      <c r="I70" s="56"/>
+      <c r="J70" s="56"/>
     </row>
     <row r="71" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B71" s="6"/>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
-      <c r="G71" s="22"/>
-      <c r="H71" s="22"/>
-      <c r="I71" s="22"/>
-      <c r="J71" s="22"/>
+      <c r="E71" s="56"/>
+      <c r="F71" s="56"/>
+      <c r="G71" s="56"/>
+      <c r="H71" s="56"/>
+      <c r="I71" s="56"/>
+      <c r="J71" s="56"/>
     </row>
     <row r="72" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B72" s="6"/>
-      <c r="E72" s="22"/>
-      <c r="F72" s="22"/>
-      <c r="G72" s="22"/>
-      <c r="H72" s="22"/>
-      <c r="I72" s="22"/>
-      <c r="J72" s="22"/>
+      <c r="E72" s="56"/>
+      <c r="F72" s="56"/>
+      <c r="G72" s="56"/>
+      <c r="H72" s="56"/>
+      <c r="I72" s="56"/>
+      <c r="J72" s="56"/>
     </row>
     <row r="73" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B73" s="6"/>
-      <c r="E73" s="22"/>
-      <c r="F73" s="22"/>
-      <c r="G73" s="22"/>
-      <c r="H73" s="22"/>
-      <c r="I73" s="22"/>
-      <c r="J73" s="22"/>
+      <c r="E73" s="56"/>
+      <c r="F73" s="56"/>
+      <c r="G73" s="56"/>
+      <c r="H73" s="56"/>
+      <c r="I73" s="56"/>
+      <c r="J73" s="56"/>
     </row>
     <row r="74" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B74" s="6"/>
-      <c r="E74" s="22"/>
-      <c r="F74" s="22"/>
-      <c r="G74" s="22"/>
-      <c r="H74" s="22"/>
-      <c r="I74" s="22"/>
-      <c r="J74" s="22"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="56"/>
+      <c r="I74" s="56"/>
+      <c r="J74" s="56"/>
     </row>
     <row r="75" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="22"/>
-      <c r="H75" s="22"/>
-      <c r="I75" s="22"/>
-      <c r="J75" s="22"/>
+      <c r="E75" s="56"/>
+      <c r="F75" s="56"/>
+      <c r="G75" s="56"/>
+      <c r="H75" s="56"/>
+      <c r="I75" s="56"/>
+      <c r="J75" s="56"/>
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B76" s="6"/>
-      <c r="E76" s="22"/>
-      <c r="F76" s="22"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="22"/>
-      <c r="I76" s="22"/>
-      <c r="J76" s="22"/>
+      <c r="E76" s="56"/>
+      <c r="F76" s="56"/>
+      <c r="G76" s="56"/>
+      <c r="H76" s="56"/>
+      <c r="I76" s="56"/>
+      <c r="J76" s="56"/>
     </row>
     <row r="77" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B77" s="6"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="22"/>
-      <c r="I77" s="22"/>
-      <c r="J77" s="22"/>
+      <c r="E77" s="56"/>
+      <c r="F77" s="56"/>
+      <c r="G77" s="56"/>
+      <c r="H77" s="56"/>
+      <c r="I77" s="56"/>
+      <c r="J77" s="56"/>
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B78" s="6"/>
-      <c r="E78" s="22"/>
-      <c r="F78" s="22"/>
-      <c r="G78" s="22"/>
-      <c r="H78" s="22"/>
-      <c r="I78" s="22"/>
-      <c r="J78" s="22"/>
+      <c r="E78" s="56"/>
+      <c r="F78" s="56"/>
+      <c r="G78" s="56"/>
+      <c r="H78" s="56"/>
+      <c r="I78" s="56"/>
+      <c r="J78" s="56"/>
     </row>
     <row r="79" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B79" s="6"/>
-      <c r="E79" s="22"/>
-      <c r="F79" s="22"/>
-      <c r="G79" s="22"/>
-      <c r="H79" s="22"/>
-      <c r="I79" s="22"/>
-      <c r="J79" s="22"/>
+      <c r="E79" s="56"/>
+      <c r="F79" s="56"/>
+      <c r="G79" s="56"/>
+      <c r="H79" s="56"/>
+      <c r="I79" s="56"/>
+      <c r="J79" s="56"/>
     </row>
     <row r="80" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B80" s="6"/>
-      <c r="E80" s="22"/>
-      <c r="F80" s="22"/>
-      <c r="G80" s="22"/>
-      <c r="H80" s="22"/>
-      <c r="I80" s="22"/>
-      <c r="J80" s="22"/>
+      <c r="E80" s="56"/>
+      <c r="F80" s="56"/>
+      <c r="G80" s="56"/>
+      <c r="H80" s="56"/>
+      <c r="I80" s="56"/>
+      <c r="J80" s="56"/>
     </row>
     <row r="81" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B81" s="6"/>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
-      <c r="G81" s="22"/>
-      <c r="H81" s="22"/>
-      <c r="I81" s="22"/>
-      <c r="J81" s="22"/>
+      <c r="E81" s="56"/>
+      <c r="F81" s="56"/>
+      <c r="G81" s="56"/>
+      <c r="H81" s="56"/>
+      <c r="I81" s="56"/>
+      <c r="J81" s="56"/>
     </row>
     <row r="82" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B82" s="6"/>
-      <c r="E82" s="22"/>
-      <c r="F82" s="22"/>
-      <c r="G82" s="22"/>
-      <c r="H82" s="22"/>
-      <c r="I82" s="22"/>
-      <c r="J82" s="22"/>
+      <c r="E82" s="56"/>
+      <c r="F82" s="56"/>
+      <c r="G82" s="56"/>
+      <c r="H82" s="56"/>
+      <c r="I82" s="56"/>
+      <c r="J82" s="56"/>
     </row>
     <row r="83" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B83" s="6"/>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="22"/>
-      <c r="H83" s="22"/>
-      <c r="I83" s="22"/>
-      <c r="J83" s="22"/>
+      <c r="E83" s="56"/>
+      <c r="F83" s="56"/>
+      <c r="G83" s="56"/>
+      <c r="H83" s="56"/>
+      <c r="I83" s="56"/>
+      <c r="J83" s="56"/>
     </row>
     <row r="84" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B84" s="6"/>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="22"/>
-      <c r="H84" s="22"/>
-      <c r="I84" s="22"/>
-      <c r="J84" s="22"/>
+      <c r="E84" s="56"/>
+      <c r="F84" s="56"/>
+      <c r="G84" s="56"/>
+      <c r="H84" s="56"/>
+      <c r="I84" s="56"/>
+      <c r="J84" s="56"/>
     </row>
     <row r="85" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B85" s="6"/>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
-      <c r="G85" s="22"/>
-      <c r="H85" s="22"/>
-      <c r="I85" s="22"/>
-      <c r="J85" s="22"/>
+      <c r="E85" s="56"/>
+      <c r="F85" s="56"/>
+      <c r="G85" s="56"/>
+      <c r="H85" s="56"/>
+      <c r="I85" s="56"/>
+      <c r="J85" s="56"/>
     </row>
     <row r="86" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B86" s="6"/>
-      <c r="E86" s="22"/>
-      <c r="F86" s="22"/>
-      <c r="G86" s="22"/>
-      <c r="H86" s="22"/>
-      <c r="I86" s="22"/>
-      <c r="J86" s="22"/>
+      <c r="E86" s="56"/>
+      <c r="F86" s="56"/>
+      <c r="G86" s="56"/>
+      <c r="H86" s="56"/>
+      <c r="I86" s="56"/>
+      <c r="J86" s="56"/>
     </row>
     <row r="87" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B87" s="6"/>
-      <c r="E87" s="22"/>
-      <c r="F87" s="22"/>
-      <c r="G87" s="22"/>
-      <c r="H87" s="22"/>
-      <c r="I87" s="22"/>
-      <c r="J87" s="22"/>
+      <c r="E87" s="56"/>
+      <c r="F87" s="56"/>
+      <c r="G87" s="56"/>
+      <c r="H87" s="56"/>
+      <c r="I87" s="56"/>
+      <c r="J87" s="56"/>
     </row>
     <row r="88" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B88" s="6"/>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
-      <c r="G88" s="22"/>
-      <c r="H88" s="22"/>
-      <c r="I88" s="22"/>
-      <c r="J88" s="22"/>
+      <c r="E88" s="56"/>
+      <c r="F88" s="56"/>
+      <c r="G88" s="56"/>
+      <c r="H88" s="56"/>
+      <c r="I88" s="56"/>
+      <c r="J88" s="56"/>
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B89" s="6"/>
-      <c r="E89" s="22"/>
-      <c r="F89" s="22"/>
-      <c r="G89" s="22"/>
-      <c r="H89" s="22"/>
-      <c r="I89" s="22"/>
-      <c r="J89" s="22"/>
+      <c r="E89" s="56"/>
+      <c r="F89" s="56"/>
+      <c r="G89" s="56"/>
+      <c r="H89" s="56"/>
+      <c r="I89" s="56"/>
+      <c r="J89" s="56"/>
     </row>
     <row r="90" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B90" s="6"/>
-      <c r="E90" s="22"/>
-      <c r="F90" s="22"/>
-      <c r="G90" s="22"/>
-      <c r="H90" s="22"/>
-      <c r="I90" s="22"/>
-      <c r="J90" s="22"/>
+      <c r="E90" s="56"/>
+      <c r="F90" s="56"/>
+      <c r="G90" s="56"/>
+      <c r="H90" s="56"/>
+      <c r="I90" s="56"/>
+      <c r="J90" s="56"/>
     </row>
     <row r="91" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B91" s="6"/>
-      <c r="E91" s="22"/>
-      <c r="F91" s="22"/>
-      <c r="G91" s="22"/>
-      <c r="H91" s="22"/>
-      <c r="I91" s="22"/>
-      <c r="J91" s="22"/>
+      <c r="E91" s="56"/>
+      <c r="F91" s="56"/>
+      <c r="G91" s="56"/>
+      <c r="H91" s="56"/>
+      <c r="I91" s="56"/>
+      <c r="J91" s="56"/>
     </row>
     <row r="92" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B92" s="6"/>
-      <c r="E92" s="22"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="22"/>
-      <c r="H92" s="22"/>
-      <c r="I92" s="22"/>
-      <c r="J92" s="22"/>
+      <c r="E92" s="56"/>
+      <c r="F92" s="56"/>
+      <c r="G92" s="56"/>
+      <c r="H92" s="56"/>
+      <c r="I92" s="56"/>
+      <c r="J92" s="56"/>
     </row>
     <row r="93" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B93" s="6"/>
-      <c r="E93" s="22"/>
-      <c r="F93" s="22"/>
-      <c r="G93" s="22"/>
-      <c r="H93" s="22"/>
-      <c r="I93" s="22"/>
-      <c r="J93" s="22"/>
+      <c r="E93" s="56"/>
+      <c r="F93" s="56"/>
+      <c r="G93" s="56"/>
+      <c r="H93" s="56"/>
+      <c r="I93" s="56"/>
+      <c r="J93" s="56"/>
     </row>
     <row r="94" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B94" s="6"/>
-      <c r="E94" s="22"/>
-      <c r="F94" s="22"/>
-      <c r="G94" s="22"/>
-      <c r="H94" s="22"/>
-      <c r="I94" s="22"/>
-      <c r="J94" s="22"/>
+      <c r="E94" s="56"/>
+      <c r="F94" s="56"/>
+      <c r="G94" s="56"/>
+      <c r="H94" s="56"/>
+      <c r="I94" s="56"/>
+      <c r="J94" s="56"/>
     </row>
     <row r="95" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B95" s="6"/>
-      <c r="E95" s="22"/>
-      <c r="F95" s="22"/>
-      <c r="G95" s="22"/>
-      <c r="H95" s="22"/>
-      <c r="I95" s="22"/>
-      <c r="J95" s="22"/>
+      <c r="E95" s="56"/>
+      <c r="F95" s="56"/>
+      <c r="G95" s="56"/>
+      <c r="H95" s="56"/>
+      <c r="I95" s="56"/>
+      <c r="J95" s="56"/>
     </row>
     <row r="96" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B96" s="6"/>
-      <c r="E96" s="22"/>
-      <c r="F96" s="22"/>
-      <c r="G96" s="22"/>
-      <c r="H96" s="22"/>
-      <c r="I96" s="22"/>
-      <c r="J96" s="22"/>
+      <c r="E96" s="56"/>
+      <c r="F96" s="56"/>
+      <c r="G96" s="56"/>
+      <c r="H96" s="56"/>
+      <c r="I96" s="56"/>
+      <c r="J96" s="56"/>
     </row>
     <row r="97" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B97" s="6"/>
-      <c r="E97" s="22"/>
-      <c r="F97" s="22"/>
-      <c r="G97" s="22"/>
-      <c r="H97" s="22"/>
-      <c r="I97" s="22"/>
-      <c r="J97" s="22"/>
+      <c r="E97" s="56"/>
+      <c r="F97" s="56"/>
+      <c r="G97" s="56"/>
+      <c r="H97" s="56"/>
+      <c r="I97" s="56"/>
+      <c r="J97" s="56"/>
     </row>
     <row r="98" spans="2:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B98" s="18" t="s">
+      <c r="B98" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="C98" s="18"/>
-      <c r="D98" s="18"/>
-      <c r="E98" s="18"/>
-      <c r="F98" s="18"/>
-      <c r="G98" s="18"/>
-      <c r="H98" s="18"/>
-      <c r="I98" s="18"/>
-      <c r="J98" s="18"/>
+      <c r="C98" s="74"/>
+      <c r="D98" s="74"/>
+      <c r="E98" s="74"/>
+      <c r="F98" s="74"/>
+      <c r="G98" s="74"/>
+      <c r="H98" s="74"/>
+      <c r="I98" s="74"/>
+      <c r="J98" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="B4:H11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:J34"/>
+    <mergeCell ref="E35:J64"/>
     <mergeCell ref="B98:J98"/>
     <mergeCell ref="B65:J65"/>
     <mergeCell ref="B66:J66"/>
     <mergeCell ref="B67:D67"/>
     <mergeCell ref="E67:J67"/>
     <mergeCell ref="E68:J97"/>
-    <mergeCell ref="B32:J32"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="E34:J34"/>
-    <mergeCell ref="E35:J64"/>
-    <mergeCell ref="B1:J1"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="B4:H11"/>
-    <mergeCell ref="B12:D12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="32" max="16838" man="1"/>
     <brk id="65" max="16838" man="1"/>
@@ -2761,1178 +2764,1216 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="68"/>
     </row>
     <row r="2" spans="2:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="35"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="71"/>
     </row>
     <row r="3" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="36"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="62" t="s">
+      <c r="C3" s="44"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="26"/>
+      <c r="J3" s="68"/>
     </row>
     <row r="4" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="58"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="28"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="48"/>
     </row>
     <row r="5" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="58"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="28"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="47"/>
+      <c r="J5" s="48"/>
     </row>
     <row r="6" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="58"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="28"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="48"/>
     </row>
     <row r="7" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="58"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="28"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="48"/>
     </row>
     <row r="8" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="58"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="63"/>
-      <c r="J8" s="28"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="47"/>
+      <c r="J8" s="48"/>
     </row>
     <row r="9" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="58"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="63"/>
-      <c r="J9" s="28"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="47"/>
+      <c r="J9" s="48"/>
     </row>
     <row r="10" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="58"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="63"/>
-      <c r="J10" s="28"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="48"/>
     </row>
     <row r="11" spans="2:10" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="58"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="29"/>
+      <c r="B11" s="59"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="50"/>
     </row>
     <row r="12" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="59" t="s">
+      <c r="B12" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="49" t="s">
+      <c r="D12" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="50"/>
-      <c r="F12" s="51" t="s">
+      <c r="E12" s="61"/>
+      <c r="F12" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="48" t="s">
+      <c r="G12" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="52" t="s">
+      <c r="H12" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="49" t="s">
+      <c r="I12" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="53"/>
+      <c r="J12" s="62"/>
     </row>
     <row r="13" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="60"/>
-      <c r="C13" s="38">
+      <c r="B13" s="31"/>
+      <c r="C13" s="14">
         <v>1</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="40"/>
-      <c r="F13" s="41">
+      <c r="E13" s="29"/>
+      <c r="F13" s="15">
         <v>490</v>
       </c>
-      <c r="G13" s="42" t="s">
+      <c r="G13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="43" t="s">
+      <c r="H13" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="54"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="52"/>
     </row>
     <row r="14" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="60"/>
-      <c r="C14" s="38">
+      <c r="B14" s="31"/>
+      <c r="C14" s="14">
         <v>2</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="40"/>
-      <c r="F14" s="45">
+      <c r="E14" s="29"/>
+      <c r="F14" s="18">
         <v>5.9</v>
       </c>
-      <c r="G14" s="42" t="s">
+      <c r="G14" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="43" t="s">
+      <c r="H14" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="54"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="52"/>
     </row>
     <row r="15" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="60"/>
-      <c r="C15" s="38">
+      <c r="B15" s="31"/>
+      <c r="C15" s="14">
         <v>3</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="40"/>
-      <c r="F15" s="45">
+      <c r="E15" s="29"/>
+      <c r="F15" s="18">
         <v>73.5</v>
       </c>
-      <c r="G15" s="42" t="s">
+      <c r="G15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="43" t="s">
+      <c r="H15" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="54"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="52"/>
     </row>
     <row r="16" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="60"/>
-      <c r="C16" s="38">
+      <c r="B16" s="31"/>
+      <c r="C16" s="14">
         <v>4</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="40"/>
-      <c r="F16" s="45">
+      <c r="E16" s="29"/>
+      <c r="F16" s="18">
         <v>98</v>
       </c>
-      <c r="G16" s="42" t="s">
+      <c r="G16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="46" t="s">
+      <c r="H16" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="54"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="52"/>
     </row>
     <row r="17" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="60"/>
-      <c r="C17" s="38">
+      <c r="B17" s="31"/>
+      <c r="C17" s="14">
         <v>5</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="40"/>
-      <c r="F17" s="45">
+      <c r="E17" s="29"/>
+      <c r="F17" s="18">
         <v>147</v>
       </c>
-      <c r="G17" s="42" t="s">
+      <c r="G17" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="46" t="s">
+      <c r="H17" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="I17" s="44"/>
-      <c r="J17" s="54"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="52"/>
     </row>
     <row r="18" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="60"/>
-      <c r="C18" s="38">
+      <c r="B18" s="31"/>
+      <c r="C18" s="14">
         <v>6</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="40"/>
-      <c r="F18" s="45">
+      <c r="E18" s="29"/>
+      <c r="F18" s="18">
         <v>227</v>
       </c>
-      <c r="G18" s="42" t="s">
+      <c r="G18" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="43" t="s">
+      <c r="H18" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="I18" s="44"/>
-      <c r="J18" s="54"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="52"/>
     </row>
     <row r="19" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="60"/>
-      <c r="C19" s="38">
+      <c r="B19" s="31"/>
+      <c r="C19" s="14">
         <v>7</v>
       </c>
-      <c r="D19" s="39"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="47"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="54"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="52"/>
     </row>
     <row r="20" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="60"/>
-      <c r="C20" s="38">
+      <c r="B20" s="31"/>
+      <c r="C20" s="14">
         <v>8</v>
       </c>
-      <c r="D20" s="39"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="54"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="52"/>
     </row>
     <row r="21" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="60"/>
-      <c r="C21" s="38">
+      <c r="B21" s="31"/>
+      <c r="C21" s="14">
         <v>9</v>
       </c>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="47"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="54"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="52"/>
     </row>
     <row r="22" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="60"/>
-      <c r="C22" s="38">
+      <c r="B22" s="31"/>
+      <c r="C22" s="14">
         <v>10</v>
       </c>
-      <c r="D22" s="39"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="54"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="52"/>
     </row>
     <row r="23" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="60"/>
-      <c r="C23" s="38">
+      <c r="B23" s="31"/>
+      <c r="C23" s="14">
         <v>11</v>
       </c>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="47"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="47"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="54"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="52"/>
     </row>
     <row r="24" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="60"/>
-      <c r="C24" s="38">
+      <c r="B24" s="31"/>
+      <c r="C24" s="14">
         <v>12</v>
       </c>
-      <c r="D24" s="39"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="54"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="52"/>
     </row>
     <row r="25" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="60"/>
-      <c r="C25" s="38">
+      <c r="B25" s="31"/>
+      <c r="C25" s="14">
         <v>13</v>
       </c>
-      <c r="D25" s="39"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="44"/>
-      <c r="J25" s="54"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="52"/>
     </row>
     <row r="26" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="60"/>
-      <c r="C26" s="38">
+      <c r="B26" s="31"/>
+      <c r="C26" s="14">
         <v>14</v>
       </c>
-      <c r="D26" s="39"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="54"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="52"/>
     </row>
     <row r="27" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="60"/>
-      <c r="C27" s="38">
+      <c r="B27" s="31"/>
+      <c r="C27" s="14">
         <v>15</v>
       </c>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="44"/>
-      <c r="J27" s="54"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="52"/>
     </row>
     <row r="28" spans="2:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="61"/>
-      <c r="C28" s="56">
+      <c r="B28" s="32"/>
+      <c r="C28" s="25">
         <v>16</v>
       </c>
-      <c r="D28" s="81"/>
-      <c r="E28" s="82"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="55"/>
-      <c r="I28" s="79"/>
-      <c r="J28" s="80"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="27"/>
     </row>
     <row r="29" spans="2:10" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="78" t="s">
+      <c r="B29" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="78"/>
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
-      <c r="F29" s="78"/>
-      <c r="G29" s="78"/>
-      <c r="H29" s="78"/>
-      <c r="I29" s="78"/>
-      <c r="J29" s="78"/>
+      <c r="C29" s="73"/>
+      <c r="D29" s="73"/>
+      <c r="E29" s="73"/>
+      <c r="F29" s="73"/>
+      <c r="G29" s="73"/>
+      <c r="H29" s="73"/>
+      <c r="I29" s="73"/>
+      <c r="J29" s="73"/>
     </row>
     <row r="30" spans="2:10" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="70" t="s">
+      <c r="B30" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71"/>
-      <c r="G30" s="71"/>
-      <c r="H30" s="71"/>
-      <c r="I30" s="71"/>
-      <c r="J30" s="72"/>
+      <c r="C30" s="64"/>
+      <c r="D30" s="64"/>
+      <c r="E30" s="64"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="64"/>
+      <c r="H30" s="64"/>
+      <c r="I30" s="64"/>
+      <c r="J30" s="65"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="73" t="s">
+      <c r="B31" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="C31" s="73"/>
-      <c r="D31" s="74"/>
-      <c r="E31" s="66" t="s">
+      <c r="C31" s="53"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="F31" s="66"/>
-      <c r="G31" s="66"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="66"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="55"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="55"/>
+      <c r="J31" s="55"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="68"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="75"/>
-      <c r="E32" s="22" t="s">
+      <c r="B32" s="33"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
+      <c r="F32" s="56"/>
+      <c r="G32" s="56"/>
+      <c r="H32" s="56"/>
+      <c r="I32" s="56"/>
+      <c r="J32" s="56"/>
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B33" s="67"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="76"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
+      <c r="G33" s="56"/>
+      <c r="H33" s="56"/>
+      <c r="I33" s="56"/>
+      <c r="J33" s="56"/>
     </row>
     <row r="34" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="67"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="56"/>
+      <c r="J34" s="56"/>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="67"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="76"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="56"/>
+      <c r="J35" s="56"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="67"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="76"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="56"/>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="67"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="76"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="56"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="67"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="76"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="37"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="56"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="67"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="76"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="67"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="76"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
+      <c r="B40" s="36"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="56"/>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B41" s="67"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="76"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
+      <c r="B41" s="36"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="56"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B42" s="67"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="76"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
+      <c r="B42" s="36"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B43" s="67"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="76"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
+      <c r="B43" s="36"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="56"/>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B44" s="67"/>
-      <c r="C44" s="27"/>
-      <c r="D44" s="76"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="22"/>
-      <c r="I44" s="22"/>
-      <c r="J44" s="22"/>
+      <c r="B44" s="36"/>
+      <c r="C44" s="37"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="56"/>
+      <c r="G44" s="56"/>
+      <c r="H44" s="56"/>
+      <c r="I44" s="56"/>
+      <c r="J44" s="56"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B45" s="67"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="76"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="56"/>
+      <c r="H45" s="56"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="56"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B46" s="67"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="76"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="37"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="56"/>
+      <c r="F46" s="56"/>
+      <c r="G46" s="56"/>
+      <c r="H46" s="56"/>
+      <c r="I46" s="56"/>
+      <c r="J46" s="56"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B47" s="67"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="76"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="22"/>
-      <c r="J47" s="22"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="37"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="56"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="56"/>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B48" s="67"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="76"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
+      <c r="B48" s="36"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="56"/>
+      <c r="J48" s="56"/>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="67"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="76"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22"/>
-      <c r="J49" s="22"/>
+      <c r="B49" s="36"/>
+      <c r="C49" s="37"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="56"/>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="67"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="76"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
+      <c r="B50" s="36"/>
+      <c r="C50" s="37"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="56"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="56"/>
+      <c r="I50" s="56"/>
+      <c r="J50" s="56"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="67"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="76"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
+      <c r="B51" s="36"/>
+      <c r="C51" s="37"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="56"/>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B52" s="67"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="76"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22"/>
-      <c r="J52" s="22"/>
+      <c r="B52" s="36"/>
+      <c r="C52" s="37"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="56"/>
+      <c r="F52" s="56"/>
+      <c r="G52" s="56"/>
+      <c r="H52" s="56"/>
+      <c r="I52" s="56"/>
+      <c r="J52" s="56"/>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B53" s="67"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="76"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
+      <c r="B53" s="36"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="38"/>
+      <c r="E53" s="56"/>
+      <c r="F53" s="56"/>
+      <c r="G53" s="56"/>
+      <c r="H53" s="56"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="56"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="67"/>
-      <c r="C54" s="27"/>
-      <c r="D54" s="76"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="22"/>
-      <c r="H54" s="22"/>
-      <c r="I54" s="22"/>
-      <c r="J54" s="22"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="56"/>
+      <c r="F54" s="56"/>
+      <c r="G54" s="56"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="56"/>
+      <c r="J54" s="56"/>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="67"/>
-      <c r="C55" s="27"/>
-      <c r="D55" s="76"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="22"/>
-      <c r="I55" s="22"/>
-      <c r="J55" s="22"/>
+      <c r="B55" s="36"/>
+      <c r="C55" s="37"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="56"/>
+      <c r="H55" s="56"/>
+      <c r="I55" s="56"/>
+      <c r="J55" s="56"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="67"/>
-      <c r="C56" s="27"/>
-      <c r="D56" s="76"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="22"/>
-      <c r="H56" s="22"/>
-      <c r="I56" s="22"/>
-      <c r="J56" s="22"/>
+      <c r="B56" s="36"/>
+      <c r="C56" s="37"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="56"/>
+      <c r="F56" s="56"/>
+      <c r="G56" s="56"/>
+      <c r="H56" s="56"/>
+      <c r="I56" s="56"/>
+      <c r="J56" s="56"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="67"/>
-      <c r="C57" s="27"/>
-      <c r="D57" s="76"/>
-      <c r="E57" s="22"/>
-      <c r="F57" s="22"/>
-      <c r="G57" s="22"/>
-      <c r="H57" s="22"/>
-      <c r="I57" s="22"/>
-      <c r="J57" s="22"/>
+      <c r="B57" s="36"/>
+      <c r="C57" s="37"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="56"/>
+      <c r="F57" s="56"/>
+      <c r="G57" s="56"/>
+      <c r="H57" s="56"/>
+      <c r="I57" s="56"/>
+      <c r="J57" s="56"/>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="67"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="76"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
-      <c r="G58" s="22"/>
-      <c r="H58" s="22"/>
-      <c r="I58" s="22"/>
-      <c r="J58" s="22"/>
+      <c r="B58" s="36"/>
+      <c r="C58" s="37"/>
+      <c r="D58" s="38"/>
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
+      <c r="I58" s="56"/>
+      <c r="J58" s="56"/>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" s="67"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="76"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
+      <c r="B59" s="36"/>
+      <c r="C59" s="37"/>
+      <c r="D59" s="38"/>
+      <c r="E59" s="56"/>
+      <c r="F59" s="56"/>
+      <c r="G59" s="56"/>
+      <c r="H59" s="56"/>
+      <c r="I59" s="56"/>
+      <c r="J59" s="56"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="67"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="76"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
+      <c r="B60" s="36"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="38"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="56"/>
+      <c r="G60" s="56"/>
+      <c r="H60" s="56"/>
+      <c r="I60" s="56"/>
+      <c r="J60" s="56"/>
     </row>
     <row r="61" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="69"/>
-      <c r="C61" s="32"/>
-      <c r="D61" s="77"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
+      <c r="B61" s="39"/>
+      <c r="C61" s="40"/>
+      <c r="D61" s="41"/>
+      <c r="E61" s="56"/>
+      <c r="F61" s="56"/>
+      <c r="G61" s="56"/>
+      <c r="H61" s="56"/>
+      <c r="I61" s="56"/>
+      <c r="J61" s="56"/>
     </row>
     <row r="62" spans="2:10" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="65" t="s">
+      <c r="B62" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="65"/>
-      <c r="D62" s="65"/>
-      <c r="E62" s="65"/>
-      <c r="F62" s="65"/>
-      <c r="G62" s="65"/>
-      <c r="H62" s="65"/>
-      <c r="I62" s="65"/>
-      <c r="J62" s="65"/>
+      <c r="C62" s="57"/>
+      <c r="D62" s="57"/>
+      <c r="E62" s="57"/>
+      <c r="F62" s="57"/>
+      <c r="G62" s="57"/>
+      <c r="H62" s="57"/>
+      <c r="I62" s="57"/>
+      <c r="J62" s="57"/>
     </row>
     <row r="63" spans="2:10" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="70" t="s">
+      <c r="B63" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C63" s="71"/>
-      <c r="D63" s="71"/>
-      <c r="E63" s="71"/>
-      <c r="F63" s="71"/>
-      <c r="G63" s="71"/>
-      <c r="H63" s="71"/>
-      <c r="I63" s="71"/>
-      <c r="J63" s="72"/>
+      <c r="C63" s="64"/>
+      <c r="D63" s="64"/>
+      <c r="E63" s="64"/>
+      <c r="F63" s="64"/>
+      <c r="G63" s="64"/>
+      <c r="H63" s="64"/>
+      <c r="I63" s="64"/>
+      <c r="J63" s="65"/>
     </row>
     <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="73" t="s">
+      <c r="B64" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="73"/>
-      <c r="D64" s="74"/>
-      <c r="E64" s="66" t="s">
+      <c r="C64" s="53"/>
+      <c r="D64" s="54"/>
+      <c r="E64" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="F64" s="66"/>
-      <c r="G64" s="66"/>
-      <c r="H64" s="66"/>
-      <c r="I64" s="66"/>
-      <c r="J64" s="66"/>
+      <c r="F64" s="55"/>
+      <c r="G64" s="55"/>
+      <c r="H64" s="55"/>
+      <c r="I64" s="55"/>
+      <c r="J64" s="55"/>
     </row>
     <row r="65" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B65" s="68"/>
-      <c r="C65" s="30"/>
-      <c r="D65" s="75"/>
-      <c r="E65" s="22" t="s">
+      <c r="B65" s="33"/>
+      <c r="C65" s="34"/>
+      <c r="D65" s="35"/>
+      <c r="E65" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="F65" s="22"/>
-      <c r="G65" s="22"/>
-      <c r="H65" s="22"/>
-      <c r="I65" s="22"/>
-      <c r="J65" s="22"/>
+      <c r="F65" s="56"/>
+      <c r="G65" s="56"/>
+      <c r="H65" s="56"/>
+      <c r="I65" s="56"/>
+      <c r="J65" s="56"/>
     </row>
     <row r="66" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B66" s="67"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="76"/>
-      <c r="E66" s="22"/>
-      <c r="F66" s="22"/>
-      <c r="G66" s="22"/>
-      <c r="H66" s="22"/>
-      <c r="I66" s="22"/>
-      <c r="J66" s="22"/>
+      <c r="B66" s="36"/>
+      <c r="C66" s="37"/>
+      <c r="D66" s="38"/>
+      <c r="E66" s="56"/>
+      <c r="F66" s="56"/>
+      <c r="G66" s="56"/>
+      <c r="H66" s="56"/>
+      <c r="I66" s="56"/>
+      <c r="J66" s="56"/>
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B67" s="67"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="76"/>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
-      <c r="G67" s="22"/>
-      <c r="H67" s="22"/>
-      <c r="I67" s="22"/>
-      <c r="J67" s="22"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="56"/>
+      <c r="F67" s="56"/>
+      <c r="G67" s="56"/>
+      <c r="H67" s="56"/>
+      <c r="I67" s="56"/>
+      <c r="J67" s="56"/>
     </row>
     <row r="68" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B68" s="67"/>
-      <c r="C68" s="27"/>
-      <c r="D68" s="76"/>
-      <c r="E68" s="22"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="22"/>
-      <c r="H68" s="22"/>
-      <c r="I68" s="22"/>
-      <c r="J68" s="22"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="37"/>
+      <c r="D68" s="38"/>
+      <c r="E68" s="56"/>
+      <c r="F68" s="56"/>
+      <c r="G68" s="56"/>
+      <c r="H68" s="56"/>
+      <c r="I68" s="56"/>
+      <c r="J68" s="56"/>
     </row>
     <row r="69" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B69" s="67"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="76"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
+      <c r="B69" s="36"/>
+      <c r="C69" s="37"/>
+      <c r="D69" s="38"/>
+      <c r="E69" s="56"/>
+      <c r="F69" s="56"/>
+      <c r="G69" s="56"/>
+      <c r="H69" s="56"/>
+      <c r="I69" s="56"/>
+      <c r="J69" s="56"/>
     </row>
     <row r="70" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B70" s="67"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="76"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="22"/>
+      <c r="B70" s="36"/>
+      <c r="C70" s="37"/>
+      <c r="D70" s="38"/>
+      <c r="E70" s="56"/>
+      <c r="F70" s="56"/>
+      <c r="G70" s="56"/>
+      <c r="H70" s="56"/>
+      <c r="I70" s="56"/>
+      <c r="J70" s="56"/>
     </row>
     <row r="71" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B71" s="67"/>
-      <c r="C71" s="27"/>
-      <c r="D71" s="76"/>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
-      <c r="G71" s="22"/>
-      <c r="H71" s="22"/>
-      <c r="I71" s="22"/>
-      <c r="J71" s="22"/>
+      <c r="B71" s="36"/>
+      <c r="C71" s="37"/>
+      <c r="D71" s="38"/>
+      <c r="E71" s="56"/>
+      <c r="F71" s="56"/>
+      <c r="G71" s="56"/>
+      <c r="H71" s="56"/>
+      <c r="I71" s="56"/>
+      <c r="J71" s="56"/>
     </row>
     <row r="72" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B72" s="67"/>
-      <c r="C72" s="27"/>
-      <c r="D72" s="76"/>
-      <c r="E72" s="22"/>
-      <c r="F72" s="22"/>
-      <c r="G72" s="22"/>
-      <c r="H72" s="22"/>
-      <c r="I72" s="22"/>
-      <c r="J72" s="22"/>
+      <c r="B72" s="36"/>
+      <c r="C72" s="37"/>
+      <c r="D72" s="38"/>
+      <c r="E72" s="56"/>
+      <c r="F72" s="56"/>
+      <c r="G72" s="56"/>
+      <c r="H72" s="56"/>
+      <c r="I72" s="56"/>
+      <c r="J72" s="56"/>
     </row>
     <row r="73" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B73" s="67"/>
-      <c r="C73" s="27"/>
-      <c r="D73" s="76"/>
-      <c r="E73" s="22"/>
-      <c r="F73" s="22"/>
-      <c r="G73" s="22"/>
-      <c r="H73" s="22"/>
-      <c r="I73" s="22"/>
-      <c r="J73" s="22"/>
+      <c r="B73" s="36"/>
+      <c r="C73" s="37"/>
+      <c r="D73" s="38"/>
+      <c r="E73" s="56"/>
+      <c r="F73" s="56"/>
+      <c r="G73" s="56"/>
+      <c r="H73" s="56"/>
+      <c r="I73" s="56"/>
+      <c r="J73" s="56"/>
     </row>
     <row r="74" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B74" s="67"/>
-      <c r="C74" s="27"/>
-      <c r="D74" s="76"/>
-      <c r="E74" s="22"/>
-      <c r="F74" s="22"/>
-      <c r="G74" s="22"/>
-      <c r="H74" s="22"/>
-      <c r="I74" s="22"/>
-      <c r="J74" s="22"/>
+      <c r="B74" s="36"/>
+      <c r="C74" s="37"/>
+      <c r="D74" s="38"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="56"/>
+      <c r="I74" s="56"/>
+      <c r="J74" s="56"/>
     </row>
     <row r="75" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B75" s="67"/>
-      <c r="C75" s="27"/>
-      <c r="D75" s="76"/>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="22"/>
-      <c r="H75" s="22"/>
-      <c r="I75" s="22"/>
-      <c r="J75" s="22"/>
+      <c r="B75" s="36"/>
+      <c r="C75" s="37"/>
+      <c r="D75" s="38"/>
+      <c r="E75" s="56"/>
+      <c r="F75" s="56"/>
+      <c r="G75" s="56"/>
+      <c r="H75" s="56"/>
+      <c r="I75" s="56"/>
+      <c r="J75" s="56"/>
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B76" s="67"/>
-      <c r="C76" s="27"/>
-      <c r="D76" s="76"/>
-      <c r="E76" s="22"/>
-      <c r="F76" s="22"/>
-      <c r="G76" s="22"/>
-      <c r="H76" s="22"/>
-      <c r="I76" s="22"/>
-      <c r="J76" s="22"/>
+      <c r="B76" s="36"/>
+      <c r="C76" s="37"/>
+      <c r="D76" s="38"/>
+      <c r="E76" s="56"/>
+      <c r="F76" s="56"/>
+      <c r="G76" s="56"/>
+      <c r="H76" s="56"/>
+      <c r="I76" s="56"/>
+      <c r="J76" s="56"/>
     </row>
     <row r="77" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B77" s="67"/>
-      <c r="C77" s="27"/>
-      <c r="D77" s="76"/>
-      <c r="E77" s="22"/>
-      <c r="F77" s="22"/>
-      <c r="G77" s="22"/>
-      <c r="H77" s="22"/>
-      <c r="I77" s="22"/>
-      <c r="J77" s="22"/>
+      <c r="B77" s="36"/>
+      <c r="C77" s="37"/>
+      <c r="D77" s="38"/>
+      <c r="E77" s="56"/>
+      <c r="F77" s="56"/>
+      <c r="G77" s="56"/>
+      <c r="H77" s="56"/>
+      <c r="I77" s="56"/>
+      <c r="J77" s="56"/>
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B78" s="67"/>
-      <c r="C78" s="27"/>
-      <c r="D78" s="76"/>
-      <c r="E78" s="22"/>
-      <c r="F78" s="22"/>
-      <c r="G78" s="22"/>
-      <c r="H78" s="22"/>
-      <c r="I78" s="22"/>
-      <c r="J78" s="22"/>
+      <c r="B78" s="36"/>
+      <c r="C78" s="37"/>
+      <c r="D78" s="38"/>
+      <c r="E78" s="56"/>
+      <c r="F78" s="56"/>
+      <c r="G78" s="56"/>
+      <c r="H78" s="56"/>
+      <c r="I78" s="56"/>
+      <c r="J78" s="56"/>
     </row>
     <row r="79" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B79" s="67"/>
-      <c r="C79" s="27"/>
-      <c r="D79" s="76"/>
-      <c r="E79" s="22"/>
-      <c r="F79" s="22"/>
-      <c r="G79" s="22"/>
-      <c r="H79" s="22"/>
-      <c r="I79" s="22"/>
-      <c r="J79" s="22"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="37"/>
+      <c r="D79" s="38"/>
+      <c r="E79" s="56"/>
+      <c r="F79" s="56"/>
+      <c r="G79" s="56"/>
+      <c r="H79" s="56"/>
+      <c r="I79" s="56"/>
+      <c r="J79" s="56"/>
     </row>
     <row r="80" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B80" s="67"/>
-      <c r="C80" s="27"/>
-      <c r="D80" s="76"/>
-      <c r="E80" s="22"/>
-      <c r="F80" s="22"/>
-      <c r="G80" s="22"/>
-      <c r="H80" s="22"/>
-      <c r="I80" s="22"/>
-      <c r="J80" s="22"/>
+      <c r="B80" s="36"/>
+      <c r="C80" s="37"/>
+      <c r="D80" s="38"/>
+      <c r="E80" s="56"/>
+      <c r="F80" s="56"/>
+      <c r="G80" s="56"/>
+      <c r="H80" s="56"/>
+      <c r="I80" s="56"/>
+      <c r="J80" s="56"/>
     </row>
     <row r="81" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B81" s="67"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="76"/>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
-      <c r="G81" s="22"/>
-      <c r="H81" s="22"/>
-      <c r="I81" s="22"/>
-      <c r="J81" s="22"/>
+      <c r="B81" s="36"/>
+      <c r="C81" s="37"/>
+      <c r="D81" s="38"/>
+      <c r="E81" s="56"/>
+      <c r="F81" s="56"/>
+      <c r="G81" s="56"/>
+      <c r="H81" s="56"/>
+      <c r="I81" s="56"/>
+      <c r="J81" s="56"/>
     </row>
     <row r="82" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B82" s="67"/>
-      <c r="C82" s="27"/>
-      <c r="D82" s="76"/>
-      <c r="E82" s="22"/>
-      <c r="F82" s="22"/>
-      <c r="G82" s="22"/>
-      <c r="H82" s="22"/>
-      <c r="I82" s="22"/>
-      <c r="J82" s="22"/>
+      <c r="B82" s="36"/>
+      <c r="C82" s="37"/>
+      <c r="D82" s="38"/>
+      <c r="E82" s="56"/>
+      <c r="F82" s="56"/>
+      <c r="G82" s="56"/>
+      <c r="H82" s="56"/>
+      <c r="I82" s="56"/>
+      <c r="J82" s="56"/>
     </row>
     <row r="83" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B83" s="67"/>
-      <c r="C83" s="27"/>
-      <c r="D83" s="76"/>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
-      <c r="G83" s="22"/>
-      <c r="H83" s="22"/>
-      <c r="I83" s="22"/>
-      <c r="J83" s="22"/>
+      <c r="B83" s="36"/>
+      <c r="C83" s="37"/>
+      <c r="D83" s="38"/>
+      <c r="E83" s="56"/>
+      <c r="F83" s="56"/>
+      <c r="G83" s="56"/>
+      <c r="H83" s="56"/>
+      <c r="I83" s="56"/>
+      <c r="J83" s="56"/>
     </row>
     <row r="84" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B84" s="67"/>
-      <c r="C84" s="27"/>
-      <c r="D84" s="76"/>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="22"/>
-      <c r="H84" s="22"/>
-      <c r="I84" s="22"/>
-      <c r="J84" s="22"/>
+      <c r="B84" s="36"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="38"/>
+      <c r="E84" s="56"/>
+      <c r="F84" s="56"/>
+      <c r="G84" s="56"/>
+      <c r="H84" s="56"/>
+      <c r="I84" s="56"/>
+      <c r="J84" s="56"/>
     </row>
     <row r="85" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B85" s="67"/>
-      <c r="C85" s="27"/>
-      <c r="D85" s="76"/>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
-      <c r="G85" s="22"/>
-      <c r="H85" s="22"/>
-      <c r="I85" s="22"/>
-      <c r="J85" s="22"/>
+      <c r="B85" s="36"/>
+      <c r="C85" s="37"/>
+      <c r="D85" s="38"/>
+      <c r="E85" s="56"/>
+      <c r="F85" s="56"/>
+      <c r="G85" s="56"/>
+      <c r="H85" s="56"/>
+      <c r="I85" s="56"/>
+      <c r="J85" s="56"/>
     </row>
     <row r="86" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B86" s="67"/>
-      <c r="C86" s="27"/>
-      <c r="D86" s="76"/>
-      <c r="E86" s="22"/>
-      <c r="F86" s="22"/>
-      <c r="G86" s="22"/>
-      <c r="H86" s="22"/>
-      <c r="I86" s="22"/>
-      <c r="J86" s="22"/>
+      <c r="B86" s="36"/>
+      <c r="C86" s="37"/>
+      <c r="D86" s="38"/>
+      <c r="E86" s="56"/>
+      <c r="F86" s="56"/>
+      <c r="G86" s="56"/>
+      <c r="H86" s="56"/>
+      <c r="I86" s="56"/>
+      <c r="J86" s="56"/>
     </row>
     <row r="87" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B87" s="67"/>
-      <c r="C87" s="27"/>
-      <c r="D87" s="76"/>
-      <c r="E87" s="22"/>
-      <c r="F87" s="22"/>
-      <c r="G87" s="22"/>
-      <c r="H87" s="22"/>
-      <c r="I87" s="22"/>
-      <c r="J87" s="22"/>
+      <c r="B87" s="36"/>
+      <c r="C87" s="37"/>
+      <c r="D87" s="38"/>
+      <c r="E87" s="56"/>
+      <c r="F87" s="56"/>
+      <c r="G87" s="56"/>
+      <c r="H87" s="56"/>
+      <c r="I87" s="56"/>
+      <c r="J87" s="56"/>
     </row>
     <row r="88" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B88" s="67"/>
-      <c r="C88" s="27"/>
-      <c r="D88" s="76"/>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
-      <c r="G88" s="22"/>
-      <c r="H88" s="22"/>
-      <c r="I88" s="22"/>
-      <c r="J88" s="22"/>
+      <c r="B88" s="36"/>
+      <c r="C88" s="37"/>
+      <c r="D88" s="38"/>
+      <c r="E88" s="56"/>
+      <c r="F88" s="56"/>
+      <c r="G88" s="56"/>
+      <c r="H88" s="56"/>
+      <c r="I88" s="56"/>
+      <c r="J88" s="56"/>
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B89" s="67"/>
-      <c r="C89" s="27"/>
-      <c r="D89" s="76"/>
-      <c r="E89" s="22"/>
-      <c r="F89" s="22"/>
-      <c r="G89" s="22"/>
-      <c r="H89" s="22"/>
-      <c r="I89" s="22"/>
-      <c r="J89" s="22"/>
+      <c r="B89" s="36"/>
+      <c r="C89" s="37"/>
+      <c r="D89" s="38"/>
+      <c r="E89" s="56"/>
+      <c r="F89" s="56"/>
+      <c r="G89" s="56"/>
+      <c r="H89" s="56"/>
+      <c r="I89" s="56"/>
+      <c r="J89" s="56"/>
     </row>
     <row r="90" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B90" s="67"/>
-      <c r="C90" s="27"/>
-      <c r="D90" s="76"/>
-      <c r="E90" s="22"/>
-      <c r="F90" s="22"/>
-      <c r="G90" s="22"/>
-      <c r="H90" s="22"/>
-      <c r="I90" s="22"/>
-      <c r="J90" s="22"/>
+      <c r="B90" s="36"/>
+      <c r="C90" s="37"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="56"/>
+      <c r="F90" s="56"/>
+      <c r="G90" s="56"/>
+      <c r="H90" s="56"/>
+      <c r="I90" s="56"/>
+      <c r="J90" s="56"/>
     </row>
     <row r="91" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B91" s="67"/>
-      <c r="C91" s="27"/>
-      <c r="D91" s="76"/>
-      <c r="E91" s="22"/>
-      <c r="F91" s="22"/>
-      <c r="G91" s="22"/>
-      <c r="H91" s="22"/>
-      <c r="I91" s="22"/>
-      <c r="J91" s="22"/>
+      <c r="B91" s="36"/>
+      <c r="C91" s="37"/>
+      <c r="D91" s="38"/>
+      <c r="E91" s="56"/>
+      <c r="F91" s="56"/>
+      <c r="G91" s="56"/>
+      <c r="H91" s="56"/>
+      <c r="I91" s="56"/>
+      <c r="J91" s="56"/>
     </row>
     <row r="92" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B92" s="67"/>
-      <c r="C92" s="27"/>
-      <c r="D92" s="76"/>
-      <c r="E92" s="22"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="22"/>
-      <c r="H92" s="22"/>
-      <c r="I92" s="22"/>
-      <c r="J92" s="22"/>
+      <c r="B92" s="36"/>
+      <c r="C92" s="37"/>
+      <c r="D92" s="38"/>
+      <c r="E92" s="56"/>
+      <c r="F92" s="56"/>
+      <c r="G92" s="56"/>
+      <c r="H92" s="56"/>
+      <c r="I92" s="56"/>
+      <c r="J92" s="56"/>
     </row>
     <row r="93" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B93" s="67"/>
-      <c r="C93" s="27"/>
-      <c r="D93" s="76"/>
-      <c r="E93" s="22"/>
-      <c r="F93" s="22"/>
-      <c r="G93" s="22"/>
-      <c r="H93" s="22"/>
-      <c r="I93" s="22"/>
-      <c r="J93" s="22"/>
+      <c r="B93" s="36"/>
+      <c r="C93" s="37"/>
+      <c r="D93" s="38"/>
+      <c r="E93" s="56"/>
+      <c r="F93" s="56"/>
+      <c r="G93" s="56"/>
+      <c r="H93" s="56"/>
+      <c r="I93" s="56"/>
+      <c r="J93" s="56"/>
     </row>
     <row r="94" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="69"/>
-      <c r="C94" s="32"/>
-      <c r="D94" s="77"/>
-      <c r="E94" s="22"/>
-      <c r="F94" s="22"/>
-      <c r="G94" s="22"/>
-      <c r="H94" s="22"/>
-      <c r="I94" s="22"/>
-      <c r="J94" s="22"/>
+      <c r="B94" s="39"/>
+      <c r="C94" s="40"/>
+      <c r="D94" s="41"/>
+      <c r="E94" s="56"/>
+      <c r="F94" s="56"/>
+      <c r="G94" s="56"/>
+      <c r="H94" s="56"/>
+      <c r="I94" s="56"/>
+      <c r="J94" s="56"/>
     </row>
     <row r="95" spans="2:10" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B95" s="65" t="s">
+      <c r="B95" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C95" s="65"/>
-      <c r="D95" s="65"/>
-      <c r="E95" s="65"/>
-      <c r="F95" s="65"/>
-      <c r="G95" s="65"/>
-      <c r="H95" s="65"/>
-      <c r="I95" s="65"/>
-      <c r="J95" s="65"/>
+      <c r="C95" s="57"/>
+      <c r="D95" s="57"/>
+      <c r="E95" s="57"/>
+      <c r="F95" s="57"/>
+      <c r="G95" s="57"/>
+      <c r="H95" s="57"/>
+      <c r="I95" s="57"/>
+      <c r="J95" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="54">
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="E64:J64"/>
+    <mergeCell ref="E65:J94"/>
+    <mergeCell ref="B95:J95"/>
+    <mergeCell ref="B3:B11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="E31:J31"/>
+    <mergeCell ref="E32:J61"/>
+    <mergeCell ref="B62:J62"/>
+    <mergeCell ref="B63:J63"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="C3:H11"/>
+    <mergeCell ref="I4:J11"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="B12:B28"/>
@@ -3949,44 +3990,6 @@
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="C3:H11"/>
-    <mergeCell ref="I4:J11"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="E64:J64"/>
-    <mergeCell ref="E65:J94"/>
-    <mergeCell ref="B95:J95"/>
-    <mergeCell ref="B3:B11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="B30:J30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E31:J31"/>
-    <mergeCell ref="E32:J61"/>
-    <mergeCell ref="B62:J62"/>
-    <mergeCell ref="B63:J63"/>
-    <mergeCell ref="B1:J1"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I19:J19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>